<commit_message>
Add story-tiles block and re-import real-patient-stories
Adds a self-contained story-tiles block: a responsive grid of patient
story tiles that expand on click to reveal the full quote/description.
Video tiles are auto-detected from a Brightcove player link and lazy-load
the embed only on click. Each tile is a keyboard-accessible button with
aria-expanded.

Re-imports the real-patient-stories page to author its 45 tiles as this
block. The prior import had flattened the tiles into broken default
content and dropped all 16 Brightcove video IDs; the new story-tiles
parser recovers them and unwraps dead javascript:void expand-anchors to
plain text while preserving real navigational links.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-patient-journey.report.xlsx
+++ b/tools/importer/reports/import-patient-journey.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="113">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,6 +61,54 @@
     <t>https://www.vyepti.com/could-vyepti-be-right-for-you</t>
   </si>
   <si>
+    <t>doctor-discussion-guide.report.json</t>
+  </si>
+  <si>
+    <t>doctor-discussion-guide</t>
+  </si>
+  <si>
+    <t>support-resources</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:23:10.563Z</t>
+  </si>
+  <si>
+    <t>Create a Discussion Guide to Navigate Your Migraine</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/doctor-discussion-guide</t>
+  </si>
+  <si>
+    <t>downloadable-resources.report.json</t>
+  </si>
+  <si>
+    <t>downloadable-resources</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:22:55.982Z</t>
+  </si>
+  <si>
+    <t>Downloadable VYEPTI® Resources for Patients</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/downloadable-resources</t>
+  </si>
+  <si>
+    <t>financial-assistance.report.json</t>
+  </si>
+  <si>
+    <t>financial-assistance</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:23:16.376Z</t>
+  </si>
+  <si>
+    <t>Financial Assistance &amp; Support for VYEPTI® (eptinezumab-jjmr)</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/financial-assistance</t>
+  </si>
+  <si>
     <t>how-vyepti-works.report.json</t>
   </si>
   <si>
@@ -100,6 +148,21 @@
     <t>https://www.vyepti.com/</t>
   </si>
   <si>
+    <t>nurse-support.report.json</t>
+  </si>
+  <si>
+    <t>nurse-support</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:23:02.293Z</t>
+  </si>
+  <si>
+    <t>Answers to VYEPTI® Questions Through VYEPTI® Nurse Support</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/nurse-support</t>
+  </si>
+  <si>
     <t>real-life-impact.report.json</t>
   </si>
   <si>
@@ -118,16 +181,115 @@
     <t>real-patient-stories.report.json</t>
   </si>
   <si>
+    <t>["story-tiles"]</t>
+  </si>
+  <si>
     <t>real-patient-stories</t>
   </si>
   <si>
-    <t>2026-06-01T18:22:44.377Z</t>
+    <t>2026-08-04T14:33:25.682Z</t>
   </si>
   <si>
     <t>Real VYEPTI® Patient Stories &amp; Reviews</t>
   </si>
   <si>
     <t>https://www.vyepti.com/real-patient-stories</t>
+  </si>
+  <si>
+    <t>share-your-migraine-story.report.json</t>
+  </si>
+  <si>
+    <t>share-your-migraine-story</t>
+  </si>
+  <si>
+    <t>engagement</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:23:38.457Z</t>
+  </si>
+  <si>
+    <t>Share Your Migraine Story With VYEPTI® (eptinezumab-jjmr)</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/share-your-migraine-story</t>
+  </si>
+  <si>
+    <t>site-map.report.json</t>
+  </si>
+  <si>
+    <t>site-map</t>
+  </si>
+  <si>
+    <t>utility</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:24:06.329Z</t>
+  </si>
+  <si>
+    <t>Site Map</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/site-map</t>
+  </si>
+  <si>
+    <t>stay-connected.report.json</t>
+  </si>
+  <si>
+    <t>stay-connected</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:23:44.508Z</t>
+  </si>
+  <si>
+    <t>Sign Up and Stay Connected With VYEPTI®</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/stay-connected</t>
+  </si>
+  <si>
+    <t>vyepti-faq.report.json</t>
+  </si>
+  <si>
+    <t>vyepti-faq</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:23:58.954Z</t>
+  </si>
+  <si>
+    <t>FAQ About VYEPTI® (eptinezumab-jjmr) Intravenous (IV) Infusion</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/vyepti-faq</t>
+  </si>
+  <si>
+    <t>vyepti-insurance-coverage.report.json</t>
+  </si>
+  <si>
+    <t>vyepti-insurance-coverage</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:23:24.171Z</t>
+  </si>
+  <si>
+    <t>Look Up Your Insurance Coverage for VYEPTI®</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/vyepti-insurance-coverage</t>
+  </si>
+  <si>
+    <t>vyepti-locator.report.json</t>
+  </si>
+  <si>
+    <t>vyepti-locator</t>
+  </si>
+  <si>
+    <t>2026-06-01T18:23:52.525Z</t>
+  </si>
+  <si>
+    <t>Find a VYEPTI® Infusion Location</t>
+  </si>
+  <si>
+    <t>https://www.vyepti.com/vyepti-locator</t>
   </si>
   <si>
     <t>vyepti-side-effects.report.json</t>
@@ -576,13 +738,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="43" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
     <col min="3" max="3" width="31" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
@@ -670,85 +832,85 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="G4" t="s">
         <v>25</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>26</v>
-      </c>
-      <c r="G4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
         <v>29</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="G5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>31</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="F6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>36</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>37</v>
-      </c>
-      <c r="H6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
         <v>39</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
       </c>
       <c r="C7" t="s">
         <v>40</v>
@@ -757,27 +919,27 @@
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
@@ -786,24 +948,24 @@
         <v>18</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -812,39 +974,299 @@
         <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>9</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
         <v>11</v>
       </c>
       <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" t="s">
+        <v>75</v>
+      </c>
+      <c r="G13" t="s">
+        <v>76</v>
+      </c>
+      <c r="H13" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" t="s">
+        <v>80</v>
+      </c>
+      <c r="G14" t="s">
+        <v>81</v>
+      </c>
+      <c r="H14" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
         <v>18</v>
       </c>
-      <c r="F10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G10" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10" t="s">
-        <v>58</v>
+      <c r="F15" t="s">
+        <v>85</v>
+      </c>
+      <c r="G15" t="s">
+        <v>86</v>
+      </c>
+      <c r="H15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" t="s">
+        <v>91</v>
+      </c>
+      <c r="H16" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>93</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
+        <v>94</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>34</v>
+      </c>
+      <c r="F17" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" t="s">
+        <v>96</v>
+      </c>
+      <c r="H17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" t="s">
+        <v>100</v>
+      </c>
+      <c r="G18" t="s">
+        <v>101</v>
+      </c>
+      <c r="H18" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19" t="s">
+        <v>106</v>
+      </c>
+      <c r="H19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
+        <v>109</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" t="s">
+        <v>110</v>
+      </c>
+      <c r="G20" t="s">
+        <v>111</v>
+      </c>
+      <c r="H20" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>